<commit_message>
updated progress report for week 4/20-4/24
</commit_message>
<xml_diff>
--- a/Progress_Report.xlsx
+++ b/Progress_Report.xlsx
@@ -6,6 +6,7 @@
     <sheet state="visible" name="Week 323 - 327" sheetId="1" r:id="rId5"/>
     <sheet state="visible" name="Week 46 - 410" sheetId="2" r:id="rId6"/>
     <sheet state="visible" name="Week 413 - 417" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name="Week 420-424" sheetId="4" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -13,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="42">
   <si>
     <t>Task</t>
   </si>
@@ -121,6 +122,24 @@
   </si>
   <si>
     <t>Waiting for how dpu will be utilized</t>
+  </si>
+  <si>
+    <t>Team Member/s</t>
+  </si>
+  <si>
+    <t>Using our fallback of movenet on the ps trying to get this working before final demo</t>
+  </si>
+  <si>
+    <t>Prateek, Madi</t>
+  </si>
+  <si>
+    <t>Top Level Python Script</t>
+  </si>
+  <si>
+    <t>Sam, Prateek</t>
+  </si>
+  <si>
+    <t>Still updating but have a functioning version</t>
   </si>
 </sst>
 </file>
@@ -214,6 +233,10 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -1084,4 +1107,234 @@
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="31.5"/>
+    <col customWidth="1" min="2" max="2" width="21.75"/>
+    <col customWidth="1" min="6" max="6" width="30.63"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>